<commit_message>
adding sample data for testing
</commit_message>
<xml_diff>
--- a/data/sample_dashboard.xlsx
+++ b/data/sample_dashboard.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Raw Data'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Raw Data'!$A$1:$L$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -367,12 +367,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$B$9:$B$13</f>
+              <f>'Summary'!$B$9:$B$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$9:$D$13</f>
+              <f>'Summary'!$D$9:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -474,12 +474,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$B$18:$B$19</f>
+              <f>'Summary'!$B$19:$B$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$18:$D$19</f>
+              <f>'Summary'!$D$19:$D$21</f>
             </numRef>
           </val>
         </ser>
@@ -528,12 +528,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'By Location'!$B$4:$B$6</f>
+              <f>'By Location'!$B$4:$B$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'By Location'!$D$4:$D$6</f>
+              <f>'By Location'!$D$4:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -631,7 +631,7 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="4320000"/>
@@ -680,8 +680,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FinOpsData" displayName="FinOpsData" ref="A1:L26" headerRowCount="1">
-  <autoFilter ref="A1:L26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FinOpsData" displayName="FinOpsData" ref="A1:L22" headerRowCount="1">
+  <autoFilter ref="A1:L22"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Subscription ID"/>
     <tableColumn id="2" name="Subscription Name"/>
@@ -989,7 +989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I20"/>
+  <dimension ref="B1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1014,7 +1014,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-29 15:54   |  Source: data/sample_costs.csv</t>
+          <t>Generated: 2026-04-29 16:41   |  Source: data/sample_009_multi_environment_costs.csv</t>
         </is>
       </c>
     </row>
@@ -1043,17 +1043,17 @@
     <row r="5" ht="36" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>$561.47</t>
+          <t>$555.91</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -1088,33 +1088,33 @@
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>databases</t>
+          <t>virtualMachines</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>285.43</v>
+        <v>300.9792</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>0.5083599864784044</v>
+        <v>0.5414149932309454</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>virtualMachines</t>
+          <t>databases</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>258.1092</v>
+        <v>248.2</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.4597007652382433</v>
+        <v>0.4464733819477249</v>
       </c>
     </row>
     <row r="11">
@@ -1124,23 +1124,23 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>17.933</v>
+        <v>6.733000000000001</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>0.03193924828335223</v>
+        <v>0.0121116248213297</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>virtualNetworks</t>
+          <t>databaseAccounts</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>0</v>
@@ -1152,11 +1152,11 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>serverFarms</t>
+          <t>components</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" s="10" t="n">
         <v>0</v>
@@ -1165,107 +1165,139 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>serverFarms</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n">
-        <v>25</v>
-      </c>
-      <c r="D14" s="18" t="n">
-        <v>561.4722</v>
-      </c>
-      <c r="E14" s="19" t="n">
+      <c r="C15" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>555.9122</v>
+      </c>
+      <c r="E15" s="19" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="6" t="inlineStr">
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cost by Subscription</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Subscription</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Resources</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Est. Cost (USD)</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>% of Total</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>356.7134</v>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>0.6353180086209077</v>
-      </c>
-    </row>
     <row r="19">
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D19" s="14" t="n">
-        <v>204.7588</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <v>0.3646819913790923</v>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Development Multi-Env</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>217.444</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>0.3911480985666442</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Production Multi-Env</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>183.4826</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0.3300567967387656</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Staging Multi-Env</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>154.9856</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>0.2787951046945902</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
-        <v>25</v>
-      </c>
-      <c r="D20" s="18" t="n">
-        <v>561.4722</v>
-      </c>
-      <c r="E20" s="19" t="n">
+      <c r="C22" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>555.9122</v>
+      </c>
+      <c r="E22" s="19" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B17:E17"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B16:E16"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="D4:E4"/>
@@ -1284,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E7"/>
+  <dimension ref="B1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1326,64 +1358,48 @@
     <row r="4">
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>westeurope</t>
+          <t>eastus</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>302.051</v>
+        <v>372.4296</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>0.5379625206733299</v>
+        <v>0.6699432032612345</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>eastus</t>
+          <t>westeurope</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>204.7588</v>
+        <v>183.4826</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>0.3646819913790923</v>
+        <v>0.3300567967387656</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>uksouth</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>54.6624</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>0.0973554879475778</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n">
-        <v>25</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>561.4722</v>
-      </c>
-      <c r="E7" s="24" t="n">
+      <c r="C6" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>555.9122</v>
+      </c>
+      <c r="E6" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1402,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1484,22 +1500,22 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>sub-dev-00a1-xxxx</t>
+          <t>sub-multienv-dev</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Development Multi-Env</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>rg-dev-compute</t>
+          <t>rg-dev-team-a</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>vm-dev-web-01</t>
+          <t>vm-dev-a-01</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -1519,7 +1535,7 @@
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Standard_D2s_v3</t>
+          <t>Standard_B2s</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
@@ -1531,31 +1547,31 @@
         <v>730</v>
       </c>
       <c r="K2" s="27" t="n">
-        <v>0.0181</v>
+        <v>0.0416</v>
       </c>
       <c r="L2" s="10" t="n">
-        <v>13.2028</v>
+        <v>30.368</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>sub-dev-00a1-xxxx</t>
+          <t>sub-multienv-dev</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Development Multi-Env</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>rg-dev-compute</t>
+          <t>rg-dev-team-a</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>vm-dev-web-02</t>
+          <t>vm-dev-a-02</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -1596,22 +1612,22 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>sub-dev-00a1-xxxx</t>
+          <t>sub-multienv-dev</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Development Multi-Env</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>rg-dev-compute</t>
+          <t>rg-dev-team-b</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>vm-dev-bastion</t>
+          <t>vm-dev-b-01</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -1652,12 +1668,12 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>sub-dev-00a1-xxxx</t>
+          <t>sub-multienv-dev</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Development Multi-Env</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -1667,7 +1683,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>stdevlogs001</t>
+          <t>stdev</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -1708,27 +1724,27 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>sub-dev-00a1-xxxx</t>
+          <t>sub-multienv-dev</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Development Multi-Env</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>rg-dev-storage</t>
+          <t>rg-dev-database</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>stdevartifacts</t>
+          <t>sqlserver-dev</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Microsoft.Storage/storageAccounts</t>
+          <t>Microsoft.Sql/servers/databases</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -1738,7 +1754,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Standard_GRS</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H6" s="25" t="inlineStr">
@@ -1752,39 +1768,39 @@
         </is>
       </c>
       <c r="J6" s="26" t="n">
-        <v>100</v>
+        <v>730</v>
       </c>
       <c r="K6" s="27" t="n">
-        <v>0.0448</v>
+        <v>0.17</v>
       </c>
       <c r="L6" s="10" t="n">
-        <v>4.48</v>
+        <v>124.1</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>sub-dev-00a1-xxxx</t>
+          <t>sub-multienv-staging</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Development</t>
+          <t>Staging Multi-Env</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>rg-dev-sql</t>
+          <t>rg-stg-compute</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>myserver-dev/app-db</t>
+          <t>vm-stg-01</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Microsoft.Sql/servers/databases</t>
+          <t>Microsoft.Compute/virtualMachines</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
@@ -1792,58 +1808,58 @@
           <t>eastus</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="inlineStr">
+      <c r="G7" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
         </is>
       </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Standard_D2s_v3</t>
+        </is>
+      </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>1 GB/Month</t>
+          <t>1 Hour</t>
         </is>
       </c>
       <c r="J7" s="28" t="n">
         <v>730</v>
       </c>
       <c r="K7" s="29" t="n">
-        <v>0.17</v>
+        <v>0.0181</v>
       </c>
       <c r="L7" s="14" t="n">
-        <v>124.1</v>
+        <v>13.2028</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>sub-dev-00a1-xxxx</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>rg-dev-web</t>
-        </is>
-      </c>
-      <c r="D8" s="30" t="inlineStr">
-        <is>
-          <t>asp-dev-api</t>
-        </is>
-      </c>
-      <c r="E8" s="30" t="inlineStr">
-        <is>
-          <t>Microsoft.Web/serverFarms</t>
-        </is>
-      </c>
-      <c r="F8" s="30" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>sub-multienv-staging</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Staging Multi-Env</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>rg-stg-compute</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>vm-stg-02</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Microsoft.Compute/virtualMachines</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>eastus</t>
         </is>
@@ -1853,167 +1869,167 @@
           <t>NDF</t>
         </is>
       </c>
-      <c r="H8" s="30" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="I8" s="30" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Standard_D2s_v3</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>1 Hour</t>
         </is>
       </c>
-      <c r="J8" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="33" t="n">
-        <v>0</v>
+      <c r="J8" s="26" t="n">
+        <v>730</v>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>0.0181</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>13.2028</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>sub-dev-00a1-xxxx</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>Development</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>rg-dev-network</t>
-        </is>
-      </c>
-      <c r="D9" s="30" t="inlineStr">
-        <is>
-          <t>vnet-dev-main</t>
-        </is>
-      </c>
-      <c r="E9" s="30" t="inlineStr">
-        <is>
-          <t>Microsoft.Network/virtualNetworks</t>
-        </is>
-      </c>
-      <c r="F9" s="30" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>sub-multienv-staging</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Staging Multi-Env</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>rg-stg-storage</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>ststg</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Microsoft.Storage/storageAccounts</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>eastus</t>
         </is>
       </c>
-      <c r="G9" s="25" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Standard_GRS</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
         </is>
       </c>
-      <c r="H9" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="I9" s="30" t="inlineStr">
-        <is>
-          <t>N/A (costs from peering/data transfer)</t>
-        </is>
-      </c>
-      <c r="J9" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="33" t="n">
-        <v>0</v>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>1 GB/Month</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="K9" s="29" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>4.48</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-staging</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Staging Multi-Env</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>rg-prod-compute-we</t>
+          <t>rg-stg-database</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>vm-prod-web-01</t>
+          <t>sqlserver-stg</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Microsoft.Compute/virtualMachines</t>
+          <t>Microsoft.Sql/servers/databases</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>westeurope</t>
-        </is>
-      </c>
-      <c r="G10" s="25" t="inlineStr">
+          <t>eastus</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Standard_D4s_v3</t>
-        </is>
-      </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>1 Hour</t>
+          <t>1 GB/Month</t>
         </is>
       </c>
       <c r="J10" s="26" t="n">
         <v>730</v>
       </c>
       <c r="K10" s="27" t="n">
-        <v>0.0444</v>
+        <v>0.17</v>
       </c>
       <c r="L10" s="10" t="n">
-        <v>32.377</v>
+        <v>124.1</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>rg-prod-compute-we</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>vm-prod-web-02</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.Compute/virtualMachines</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>westeurope</t>
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>sub-multienv-staging</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Staging Multi-Env</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>rg-stg-web</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>asp-stg</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>Microsoft.Web/serverFarms</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>eastus</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
@@ -2021,45 +2037,45 @@
           <t>NDF</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>Standard_D4s_v3</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
         <is>
           <t>1 Hour</t>
         </is>
       </c>
-      <c r="J11" s="28" t="n">
-        <v>730</v>
-      </c>
-      <c r="K11" s="29" t="n">
-        <v>0.0444</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>32.377</v>
+      <c r="J11" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>rg-prod-compute-we</t>
+          <t>rg-prod-web-team</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>vm-prod-web-03</t>
+          <t>vm-prod-web-01</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -2100,22 +2116,22 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>rg-prod-compute-we</t>
+          <t>rg-prod-web-team</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>vm-prod-api-01</t>
+          <t>vm-prod-web-02</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -2135,7 +2151,7 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>Standard_D2s_v3</t>
+          <t>Standard_D4s_v3</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
@@ -2147,31 +2163,31 @@
         <v>730</v>
       </c>
       <c r="K13" s="29" t="n">
-        <v>0.0222</v>
+        <v>0.0444</v>
       </c>
       <c r="L13" s="14" t="n">
-        <v>16.1885</v>
+        <v>32.377</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>rg-prod-compute-we</t>
+          <t>rg-prod-web-team</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>vm-prod-api-02</t>
+          <t>vm-prod-web-03</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -2191,7 +2207,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Standard_D2s_v3</t>
+          <t>Standard_D4s_v3</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -2203,31 +2219,31 @@
         <v>730</v>
       </c>
       <c r="K14" s="27" t="n">
-        <v>0.0222</v>
+        <v>0.0444</v>
       </c>
       <c r="L14" s="10" t="n">
-        <v>16.1885</v>
+        <v>32.377</v>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>rg-prod-compute-uks</t>
+          <t>rg-prod-api-team</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>vm-prod-db-01</t>
+          <t>vm-prod-api-01</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -2237,7 +2253,7 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>uksouth</t>
+          <t>westeurope</t>
         </is>
       </c>
       <c r="G15" s="25" t="inlineStr">
@@ -2259,31 +2275,31 @@
         <v>730</v>
       </c>
       <c r="K15" s="29" t="n">
-        <v>0.0374</v>
+        <v>0.0591</v>
       </c>
       <c r="L15" s="14" t="n">
-        <v>27.3312</v>
+        <v>43.1693</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>rg-prod-compute-uks</t>
+          <t>rg-prod-api-team</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>vm-prod-db-02</t>
+          <t>vm-prod-api-02</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -2293,7 +2309,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>uksouth</t>
+          <t>westeurope</t>
         </is>
       </c>
       <c r="G16" s="25" t="inlineStr">
@@ -2315,21 +2331,21 @@
         <v>730</v>
       </c>
       <c r="K16" s="27" t="n">
-        <v>0.0374</v>
+        <v>0.0591</v>
       </c>
       <c r="L16" s="10" t="n">
-        <v>27.3312</v>
+        <v>43.1693</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -2339,7 +2355,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>stprodlogs001</t>
+          <t>stprod</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -2354,7 +2370,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>Standard_GRS</t>
+          <t>Premium_LRS</t>
         </is>
       </c>
       <c r="H17" s="25" t="inlineStr">
@@ -2364,53 +2380,53 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>1 GB/Month</t>
+          <t>1 GiB/Hour</t>
         </is>
       </c>
       <c r="J17" s="28" t="n">
         <v>100</v>
       </c>
       <c r="K17" s="29" t="n">
-        <v>0.0448</v>
+        <v>0.0001</v>
       </c>
       <c r="L17" s="14" t="n">
-        <v>4.48</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>rg-prod-storage</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>stprodbackups</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Microsoft.Storage/storageAccounts</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>sub-multienv-prod</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Production Multi-Env</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>rg-prod-database</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>sqlserver-prod</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>Microsoft.Sql/servers/databases</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
         <is>
           <t>westeurope</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Standard_GRS</t>
+      <c r="G18" s="30" t="inlineStr">
+        <is>
+          <t>GeneralPurpose</t>
         </is>
       </c>
       <c r="H18" s="25" t="inlineStr">
@@ -2418,157 +2434,157 @@
           <t>NDF</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>1 GB/Month</t>
-        </is>
-      </c>
-      <c r="J18" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="K18" s="27" t="n">
-        <v>0.0448</v>
-      </c>
-      <c r="L18" s="10" t="n">
-        <v>4.48</v>
+      <c r="I18" s="30" t="inlineStr">
+        <is>
+          <t>1 Hour</t>
+        </is>
+      </c>
+      <c r="J18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>rg-prod-storage</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>stprodstatic</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.Storage/storageAccounts</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>sub-multienv-prod</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Production Multi-Env</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>rg-prod-database</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>cosmosdb-prod</t>
+        </is>
+      </c>
+      <c r="E19" s="30" t="inlineStr">
+        <is>
+          <t>Microsoft.DocumentDB/databaseAccounts</t>
+        </is>
+      </c>
+      <c r="F19" s="30" t="inlineStr">
         <is>
           <t>westeurope</t>
         </is>
       </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>Standard_LRS</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="inlineStr">
+      <c r="G19" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
         </is>
       </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>1 GB/Month</t>
-        </is>
-      </c>
-      <c r="J19" s="28" t="n">
-        <v>100</v>
-      </c>
-      <c r="K19" s="29" t="n">
-        <v>0.0224</v>
-      </c>
-      <c r="L19" s="14" t="n">
-        <v>2.24</v>
+      <c r="H19" s="30" t="inlineStr">
+        <is>
+          <t>Multi-region</t>
+        </is>
+      </c>
+      <c r="I19" s="30" t="inlineStr">
+        <is>
+          <t>Unsupported type</t>
+        </is>
+      </c>
+      <c r="J19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>rg-prod-storage</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>stprodpremium</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Microsoft.Storage/storageAccounts</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>sub-multienv-prod</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Production Multi-Env</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>rg-prod-web</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>asp-prod-main</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>Microsoft.Web/serverFarms</t>
+        </is>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
         <is>
           <t>westeurope</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Premium_LRS</t>
-        </is>
-      </c>
-      <c r="H20" s="25" t="inlineStr">
+      <c r="G20" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>1 GiB/Hour</t>
-        </is>
-      </c>
-      <c r="J20" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="K20" s="27" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="L20" s="10" t="n">
-        <v>0.013</v>
+      <c r="H20" s="30" t="inlineStr">
+        <is>
+          <t>P2v2</t>
+        </is>
+      </c>
+      <c r="I20" s="30" t="inlineStr">
+        <is>
+          <t>1 Hour</t>
+        </is>
+      </c>
+      <c r="J20" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="30" t="inlineStr">
         <is>
-          <t>sub-prod-00b2-xxxx</t>
+          <t>sub-multienv-prod</t>
         </is>
       </c>
       <c r="B21" s="30" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Production Multi-Env</t>
         </is>
       </c>
       <c r="C21" s="30" t="inlineStr">
         <is>
-          <t>rg-prod-sql</t>
+          <t>rg-prod-web</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>myserver-prod/orders-db</t>
+          <t>asp-prod-api</t>
         </is>
       </c>
       <c r="E21" s="30" t="inlineStr">
         <is>
-          <t>Microsoft.Sql/servers/databases</t>
+          <t>Microsoft.Web/serverFarms</t>
         </is>
       </c>
       <c r="F21" s="30" t="inlineStr">
@@ -2576,14 +2592,14 @@
           <t>westeurope</t>
         </is>
       </c>
-      <c r="G21" s="30" t="inlineStr">
-        <is>
-          <t>GeneralPurpose</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="inlineStr">
+      <c r="G21" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
+        </is>
+      </c>
+      <c r="H21" s="30" t="inlineStr">
+        <is>
+          <t>P2v2</t>
         </is>
       </c>
       <c r="I21" s="30" t="inlineStr">
@@ -2602,287 +2618,63 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>rg-prod-sql</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>myserver-prod/analytics-db</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Microsoft.Sql/servers/databases</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>sub-multienv-prod</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Production Multi-Env</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>rg-prod-insights</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>appinsights-prod</t>
+        </is>
+      </c>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>Microsoft.Insights/components</t>
+        </is>
+      </c>
+      <c r="F22" s="30" t="inlineStr">
         <is>
           <t>westeurope</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="H22" s="25" t="inlineStr">
+      <c r="G22" s="25" t="inlineStr">
         <is>
           <t>NDF</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>1 GB/Month</t>
-        </is>
-      </c>
-      <c r="J22" s="26" t="n">
-        <v>730</v>
-      </c>
-      <c r="K22" s="27" t="n">
-        <v>0.221</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>161.33</v>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t>rg-prod-web</t>
-        </is>
-      </c>
-      <c r="D23" s="30" t="inlineStr">
-        <is>
-          <t>asp-prod-main</t>
-        </is>
-      </c>
-      <c r="E23" s="30" t="inlineStr">
-        <is>
-          <t>Microsoft.Web/serverFarms</t>
-        </is>
-      </c>
-      <c r="F23" s="30" t="inlineStr">
-        <is>
-          <t>westeurope</t>
-        </is>
-      </c>
-      <c r="G23" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="H23" s="30" t="inlineStr">
-        <is>
-          <t>P2v2</t>
-        </is>
-      </c>
-      <c r="I23" s="30" t="inlineStr">
-        <is>
-          <t>1 Hour</t>
-        </is>
-      </c>
-      <c r="J23" s="31" t="n">
+      <c r="H22" s="30" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="I22" s="30" t="inlineStr">
+        <is>
+          <t>Unsupported type</t>
+        </is>
+      </c>
+      <c r="J22" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="32" t="n">
+      <c r="K22" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="33" t="n">
+      <c r="L22" s="33" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C24" s="30" t="inlineStr">
-        <is>
-          <t>rg-prod-web</t>
-        </is>
-      </c>
-      <c r="D24" s="30" t="inlineStr">
-        <is>
-          <t>asp-prod-api</t>
-        </is>
-      </c>
-      <c r="E24" s="30" t="inlineStr">
-        <is>
-          <t>Microsoft.Web/serverFarms</t>
-        </is>
-      </c>
-      <c r="F24" s="30" t="inlineStr">
-        <is>
-          <t>eastus</t>
-        </is>
-      </c>
-      <c r="G24" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="H24" s="30" t="inlineStr">
-        <is>
-          <t>P1v2</t>
-        </is>
-      </c>
-      <c r="I24" s="30" t="inlineStr">
-        <is>
-          <t>1 Hour</t>
-        </is>
-      </c>
-      <c r="J24" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t>rg-prod-network</t>
-        </is>
-      </c>
-      <c r="D25" s="30" t="inlineStr">
-        <is>
-          <t>vnet-prod-westeurope</t>
-        </is>
-      </c>
-      <c r="E25" s="30" t="inlineStr">
-        <is>
-          <t>Microsoft.Network/virtualNetworks</t>
-        </is>
-      </c>
-      <c r="F25" s="30" t="inlineStr">
-        <is>
-          <t>westeurope</t>
-        </is>
-      </c>
-      <c r="G25" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="I25" s="30" t="inlineStr">
-        <is>
-          <t>N/A (costs from peering/data transfer)</t>
-        </is>
-      </c>
-      <c r="J25" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>sub-prod-00b2-xxxx</t>
-        </is>
-      </c>
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="C26" s="30" t="inlineStr">
-        <is>
-          <t>rg-prod-network</t>
-        </is>
-      </c>
-      <c r="D26" s="30" t="inlineStr">
-        <is>
-          <t>vnet-prod-uksouth</t>
-        </is>
-      </c>
-      <c r="E26" s="30" t="inlineStr">
-        <is>
-          <t>Microsoft.Network/virtualNetworks</t>
-        </is>
-      </c>
-      <c r="F26" s="30" t="inlineStr">
-        <is>
-          <t>uksouth</t>
-        </is>
-      </c>
-      <c r="G26" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="H26" s="25" t="inlineStr">
-        <is>
-          <t>NDF</t>
-        </is>
-      </c>
-      <c r="I26" s="30" t="inlineStr">
-        <is>
-          <t>N/A (costs from peering/data transfer)</t>
-        </is>
-      </c>
-      <c r="J26" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L26"/>
+  <autoFilter ref="A1:L22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>